<commit_message>
using regex the exact phone number is extracted
</commit_message>
<xml_diff>
--- a/Software_Houses_in_Johar_Town_Lahore_lead.xlsx
+++ b/Software_Houses_in_Johar_Town_Lahore_lead.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -463,31 +463,31 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Open 24 hours · +92 318 0910776</t>
+          <t>+92 318 0910776</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Pixelpk Technologies</t>
+          <t>724.ONE (pvt) ltd</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>724.ONE (pvt) ltd</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Open · Closes 8 PM · +92 300 1181947</t>
+          <t>+92 324 6165462</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>NorthBay Solutions</t>
+          <t>Programmers Force</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -497,14 +497,14 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Closed · Opens 9 AM Mon · +92 42 35290154</t>
+          <t>+92 309 5552608</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Programmers Force</t>
+          <t>Techesthete</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -514,31 +514,31 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Closed · Opens 9 AM Mon · +92 309 5552608</t>
+          <t>+92 321 6955844</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>724.ONE (pvt) ltd</t>
+          <t>IT Genesis -- The Best Softwar</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>724.ONE (pvt) ltd</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Closed · Opens 10 AM Mon · +92 324 6165462</t>
+          <t>+92 301 9105640</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Logictex IT Solutions</t>
+          <t>DeskZone</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -548,14 +548,14 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Open · Closes 12 AM · +61 427 428 181</t>
+          <t>+1 832-253-0532</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Spadasoft Software Development</t>
+          <t>NorthBay Solutions</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -565,14 +565,14 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Closed · Opens 10 AM Mon · +92 325 1041041</t>
+          <t>+92 42 35290154</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Funzoft Pvt. Ltd.</t>
+          <t>Pixelpk Technologies</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -582,14 +582,14 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Closes soon · 6 PM · Opens 9 AM Mon · +92 303 2026650</t>
+          <t>+92 300 1181947</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Devbunch Private Limited</t>
+          <t>Spadasoft Software Development</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -599,7 +599,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Closed · Opens 9 AM Mon · +92 309 4010099</t>
+          <t>+92 325 1041041</t>
         </is>
       </c>
     </row>
@@ -616,14 +616,14 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Closed · Opens 12 AM Mon · +92 313 4732161</t>
+          <t>+92 313 4732161</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tecnomics International (Pvt) </t>
+          <t>Olumi Tech - Lahore software h</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -633,14 +633,14 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Closed · Opens 11 AM Mon · +92 42 35291920</t>
+          <t>+92 316 8844669</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>𝐒𝐭𝐚𝐜𝐤𝐬𝐌𝐢𝐧𝐝 𝐓𝐞𝐜𝐡𝐧𝐨𝐥𝐨𝐠𝐢𝐞𝐬</t>
+          <t>Synavos</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -650,14 +650,14 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Open · Closes 12 AM · +92 312 4554506</t>
+          <t>+92 42 35445651</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>OptimaGeeks</t>
+          <t>BrainX Technologies</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -667,14 +667,14 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Closed · Opens 9:30 AM Mon · +92 300 1122805</t>
+          <t>+92 42 38913038</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Nisum Pakistan (Pvt.) Ltd.</t>
+          <t>HORIZAM</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -684,14 +684,14 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Closed · Opens 9 AM Mon · +92 304 4526221</t>
+          <t>+92 42 35136201</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Nextbridge Ltd.</t>
+          <t>Funzoft Pvt. Ltd.</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -701,14 +701,14 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Closed · Opens 8 AM Mon · +92 42 35315043</t>
+          <t>+92 303 2026650</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Synavos</t>
+          <t>Viral Square</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -718,14 +718,14 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Closed · Opens 9 AM Mon · +92 42 35445651</t>
+          <t>+92 305 4444052</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>OptimusFox (Pvt.) Ltd. | Block</t>
+          <t>Devbunch Private Limited</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -735,14 +735,14 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Closed · Opens 10 AM Mon · +92 310 8881606</t>
+          <t>+92 309 4010099</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>InvoZone</t>
+          <t>AllZone Technologies</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -752,14 +752,14 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Closed · Opens 9 AM Mon · +92 317 7711171</t>
+          <t>+92 301 4786262</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Intelliscence - Software Devel</t>
+          <t>Software Alliance</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -769,14 +769,14 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Closed · Opens 9 AM Mon · +92 345 4090775</t>
+          <t>+92 300 9794063</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Developers Studio</t>
+          <t>OptimusFox (Pvt.) Ltd. | Block</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -786,160 +786,143 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Closed · Opens 9 AM Mon · +92 326 4012756</t>
+          <t>+92 310 8881606</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Software Alliance</t>
+          <t xml:space="preserve">Tecnomics International (Pvt) </t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>4.5(47)</t>
+          <t>4.0(30)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Closed · Opens 10 AM Mon · +92 300 9794063</t>
+          <t>+92 42 35291920</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>DevFactori</t>
+          <t>Digital Aims</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>4.5(46)</t>
+          <t>5.0(3)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Closed · Opens 9 AM Mon · +92 42 38347336</t>
+          <t>+92 300 2302063</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>AllZone Technologies</t>
+          <t>OptimaGeeks</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>4.6(22)</t>
+          <t>4.6(35)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Closed · Opens 1 PM Mon · +92 301 4786262</t>
+          <t>+92 300 1122805</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>BrainBox Technologies</t>
+          <t>Teknohus</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>4.9(13)</t>
+          <t>4.5(98)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Closed · Opens 12 AM Mon · +44 7966 657481</t>
+          <t>+92 42 35211702</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>IIFA TECH</t>
+          <t>Narsun Studios Pakistan</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>5.0(102)</t>
+          <t>4.4(108)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Software company · Ali Ibn-e-Abi Talib Rd</t>
+          <t>+92 323 8996619</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Nodlays</t>
+          <t>KeyDevs Technologies Pvt. Ltd.</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>4.9(17)</t>
+          <t>4.5(22)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Closed · Opens 10 AM Mon · +92 42 35136413</t>
+          <t>+92 42 35173340</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>HORIZAM</t>
+          <t>Xint Solutions</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>4.9(15)</t>
+          <t>4.7(33)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Closed · Opens 10 AM Mon · +92 42 35136201</t>
+          <t>+92 42 35301168</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Viral Square</t>
+          <t>InvoZone</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>4.1(63)</t>
+          <t>4.6(108)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Closed · Opens 12 AM Mon · +92 305 4444052</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>DeskZone</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>4.5(24)</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Open 24 hours · +1 832-253-0532</t>
+          <t>+92 317 7711171</t>
         </is>
       </c>
     </row>

</xml_diff>